<commit_message>
uploaded on date 03-03-2026
</commit_message>
<xml_diff>
--- a/Icaffe_TestCases_Tracker_Log.xlsx
+++ b/Icaffe_TestCases_Tracker_Log.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="90">
   <si>
     <t>SL No.</t>
   </si>
@@ -77,9 +77,6 @@
     <t>Masters</t>
   </si>
   <si>
-    <t>Party --&gt; Bank BRO</t>
-  </si>
-  <si>
     <t>Shivam Singh</t>
   </si>
   <si>
@@ -89,78 +86,24 @@
     <t>Pending</t>
   </si>
   <si>
-    <t>Page Responsiveness and Session Timeout test cases are currently on hold.</t>
-  </si>
-  <si>
     <t>Sudhir kumar sinha</t>
   </si>
   <si>
-    <t>Party --&gt; CFS Master</t>
-  </si>
-  <si>
-    <t>EDI Master --&gt; Currency</t>
-  </si>
-  <si>
     <t>Suraj Rana</t>
   </si>
   <si>
     <t>Done</t>
   </si>
   <si>
-    <t>EDI Master --&gt; RITC</t>
-  </si>
-  <si>
-    <t>EDI Master --&gt; Port</t>
-  </si>
-  <si>
-    <t>Regional Master --&gt; Zone Master</t>
-  </si>
-  <si>
-    <t>Regional Master --&gt; Country Master</t>
-  </si>
-  <si>
-    <t>Regional Master --&gt; Region Master</t>
-  </si>
-  <si>
-    <t>Regional Master --&gt; FF Port Master</t>
-  </si>
-  <si>
-    <t>Regional Master --&gt; Action Master</t>
-  </si>
-  <si>
-    <t>Regional Master --&gt; Period Master</t>
-  </si>
-  <si>
     <t>Regional Master --&gt; Cost Center Master</t>
   </si>
   <si>
-    <t>Shipment info --&gt; IMO Master</t>
-  </si>
-  <si>
-    <t>Shipment info --&gt; Unit Master</t>
-  </si>
-  <si>
-    <t>Shipment info --&gt; CHA Service</t>
-  </si>
-  <si>
-    <t>Misc Master - Trigger Master</t>
-  </si>
-  <si>
     <t>Misc Master - Pricniple Line HBL Master</t>
   </si>
   <si>
-    <t>Misc Master - Project Type Master</t>
-  </si>
-  <si>
     <t>Misc Master - Notes, Terms &amp; Conditions</t>
   </si>
   <si>
-    <t>Vessel Info - Vessel</t>
-  </si>
-  <si>
-    <t>Vessel Info - Schedule</t>
-  </si>
-  <si>
     <t xml:space="preserve">Misc Master - Segment Master
 </t>
   </si>
@@ -197,10 +140,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Activity
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Charge Master - Pricing
 </t>
   </si>
@@ -216,9 +155,6 @@
 </t>
   </si>
   <si>
-    <t>EDI Master --&gt; Loading &amp; CHA Port</t>
-  </si>
-  <si>
     <t>BA-482</t>
   </si>
   <si>
@@ -275,9 +211,6 @@
     <t>BA-656</t>
   </si>
   <si>
-    <t>Hold</t>
-  </si>
-  <si>
     <t xml:space="preserve">EDI Master --&gt; Item Template Master
 </t>
   </si>
@@ -297,14 +230,110 @@
 </t>
   </si>
   <si>
-    <t>Master</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ledger Account
-</t>
-  </si>
-  <si>
     <t>Working</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Party --&gt; Bank BRO
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Party --&gt; CFS Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDI Master --&gt; Currency
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDI Master --&gt; RITC
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDI Master --&gt; Port
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDI Master --&gt; Loading &amp; CHA Port
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regional Master --&gt; Zone Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regional Master --&gt; Country Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regional Master --&gt; Region Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regional Master --&gt; FF Port Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regional Master --&gt; Action Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regional Master --&gt; Period Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipment info --&gt; IMO Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipment info --&gt; Unit Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipment info --&gt; CHA Service
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misc Master - Trigger Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misc Master - Project Type Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vessel Info - Vessel
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vessel Info - Schedule
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipment Plan Master
+</t>
+  </si>
+  <si>
+    <t>Accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; Ledger Account
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; GST Charges
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipment Plan -&gt; Shipment Plan
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; TDS Schedule
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; Charge Rules
+</t>
   </si>
 </sst>
 </file>
@@ -892,7 +921,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T49"/>
+  <dimension ref="A1:T53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="18"/>
@@ -977,10 +1006,10 @@
         <v>18</v>
       </c>
       <c r="T1" s="42" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" ht="30">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="31.5">
       <c r="A2" s="19">
         <v>1</v>
       </c>
@@ -988,20 +1017,18 @@
         <v>19</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="D2" s="8">
         <v>55</v>
       </c>
       <c r="E2" s="8">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F2" s="8">
         <v>13</v>
       </c>
-      <c r="G2" s="8">
-        <v>2</v>
-      </c>
+      <c r="G2" s="8"/>
       <c r="H2" s="8">
         <v>13</v>
       </c>
@@ -1009,7 +1036,7 @@
         <v>13</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K2" s="10">
         <v>45968</v>
@@ -1018,28 +1045,26 @@
         <v>46045</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O2" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O2" s="26"/>
       <c r="P2" s="9"/>
       <c r="Q2" s="12" t="str">
         <f>HYPERLINK("#'Bank_BRO'!A1","Bank_BRO")</f>
         <v>Bank_BRO</v>
       </c>
       <c r="R2" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S2" s="26"/>
       <c r="T2" s="7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" ht="30">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" ht="31.5">
       <c r="A3" s="20">
         <v>2</v>
       </c>
@@ -1047,20 +1072,18 @@
         <v>19</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="D3" s="8">
         <v>75</v>
       </c>
       <c r="E3" s="8">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F3" s="8">
         <v>30</v>
       </c>
-      <c r="G3" s="8">
-        <v>2</v>
-      </c>
+      <c r="G3" s="8"/>
       <c r="H3" s="8">
         <v>30</v>
       </c>
@@ -1068,7 +1091,7 @@
         <v>30</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K3" s="10">
         <v>45975</v>
@@ -1077,28 +1100,26 @@
         <v>46034</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O3" s="11"/>
       <c r="P3" s="9"/>
       <c r="Q3" s="12" t="str">
         <f>HYPERLINK("#'CFS Master'!A1","CFS Master")</f>
         <v>CFS Master</v>
       </c>
       <c r="R3" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S3" s="21"/>
       <c r="T3" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" ht="30">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="31.5">
       <c r="A4" s="20">
         <v>3</v>
       </c>
@@ -1106,20 +1127,18 @@
         <v>19</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="D4" s="8">
         <v>29</v>
       </c>
       <c r="E4" s="8">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F4" s="8">
         <v>2</v>
       </c>
-      <c r="G4" s="8">
-        <v>2</v>
-      </c>
+      <c r="G4" s="8"/>
       <c r="H4" s="8">
         <v>2</v>
       </c>
@@ -1127,7 +1146,7 @@
         <v>2</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K4" s="10">
         <v>45983</v>
@@ -1136,28 +1155,26 @@
         <v>46028</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O4" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O4" s="26"/>
       <c r="P4" s="9"/>
       <c r="Q4" s="12" t="str">
         <f>HYPERLINK("#'Currency'!A1","Currency")</f>
         <v>Currency</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S4" s="21"/>
       <c r="T4" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" ht="30">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" ht="31.5">
       <c r="A5" s="20">
         <v>4</v>
       </c>
@@ -1165,20 +1182,18 @@
         <v>19</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="D5" s="8">
         <v>29</v>
       </c>
       <c r="E5" s="8">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F5" s="8">
         <v>10</v>
       </c>
-      <c r="G5" s="8">
-        <v>2</v>
-      </c>
+      <c r="G5" s="8"/>
       <c r="H5" s="8">
         <v>10</v>
       </c>
@@ -1186,7 +1201,7 @@
         <v>10</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K5" s="10">
         <v>45986</v>
@@ -1195,28 +1210,26 @@
         <v>46055</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O5" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O5" s="26"/>
       <c r="P5" s="9"/>
       <c r="Q5" s="12" t="str">
         <f>HYPERLINK("#'RITC'!A1","RITC")</f>
         <v>RITC</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S5" s="21"/>
       <c r="T5" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" ht="30">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" ht="31.5">
       <c r="A6" s="22">
         <v>5</v>
       </c>
@@ -1224,26 +1237,24 @@
         <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="D6" s="2">
         <v>21</v>
       </c>
       <c r="E6" s="2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2">
         <v>7</v>
       </c>
-      <c r="G6" s="2">
-        <v>2</v>
-      </c>
+      <c r="G6" s="2"/>
       <c r="H6" s="2">
         <v>7</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K6" s="4">
         <v>45990</v>
@@ -1251,23 +1262,21 @@
       <c r="L6" s="23"/>
       <c r="M6" s="23"/>
       <c r="N6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O6" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O6" s="7"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="6" t="str">
         <f>HYPERLINK("#'Port'!A1","Port")</f>
         <v>Port</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S6" s="23"/>
       <c r="T6" s="25"/>
     </row>
-    <row r="7" spans="1:20" ht="30">
+    <row r="7" spans="1:20" ht="31.5">
       <c r="A7" s="22">
         <v>6</v>
       </c>
@@ -1275,7 +1284,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D7" s="2">
         <v>0</v>
@@ -1286,29 +1295,27 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="23"/>
       <c r="M7" s="23"/>
       <c r="N7" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O7" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O7" s="7"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="6" t="str">
         <f>HYPERLINK("#'Loading &amp; CHA Port'!A1","Loading &amp; CHA Port")</f>
         <v>Loading &amp; CHA Port</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S7" s="23"/>
       <c r="T7" s="25"/>
     </row>
-    <row r="8" spans="1:20" ht="30">
+    <row r="8" spans="1:20" ht="31.5">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -1316,20 +1323,18 @@
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="D8" s="8">
         <v>20</v>
       </c>
       <c r="E8" s="8">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F8" s="8">
         <v>5</v>
       </c>
-      <c r="G8" s="8">
-        <v>2</v>
-      </c>
+      <c r="G8" s="8"/>
       <c r="H8" s="8">
         <v>5</v>
       </c>
@@ -1337,7 +1342,7 @@
         <v>5</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K8" s="10">
         <v>45992</v>
@@ -1346,83 +1351,81 @@
         <v>46035</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O8" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O8" s="26"/>
       <c r="P8" s="9"/>
       <c r="Q8" s="12" t="str">
         <f>HYPERLINK("#'Zone Master'!A1","Zone Master")</f>
         <v>Zone Master</v>
       </c>
       <c r="R8" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S8" s="11"/>
       <c r="T8" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" ht="30">
-      <c r="A9" s="44">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" ht="31.5">
+      <c r="A9" s="20">
         <v>8</v>
       </c>
-      <c r="B9" s="45" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="45">
+      <c r="B9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="8">
         <v>25</v>
       </c>
-      <c r="E9" s="45">
-        <v>15</v>
-      </c>
-      <c r="F9" s="45">
+      <c r="E9" s="8">
+        <v>17</v>
+      </c>
+      <c r="F9" s="8">
         <v>8</v>
       </c>
-      <c r="G9" s="45">
-        <v>2</v>
-      </c>
-      <c r="H9" s="45">
+      <c r="G9" s="8"/>
+      <c r="H9" s="8">
         <v>8</v>
       </c>
-      <c r="I9" s="45">
+      <c r="I9" s="8">
         <v>8</v>
       </c>
-      <c r="J9" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="K9" s="46">
+      <c r="J9" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" s="10">
         <v>45992</v>
       </c>
-      <c r="L9" s="46"/>
-      <c r="M9" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="N9" s="46" t="s">
-        <v>29</v>
-      </c>
-      <c r="O9" s="47" t="s">
+      <c r="L9" s="10">
+        <v>46079</v>
+      </c>
+      <c r="M9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="P9" s="45"/>
-      <c r="Q9" s="48" t="str">
+      <c r="N9" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O9" s="26"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="12" t="str">
         <f>HYPERLINK("#'Country Master'!A1","Country Master")</f>
         <v>Country Master</v>
       </c>
-      <c r="R9" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="S9" s="49"/>
-      <c r="T9" s="7"/>
-    </row>
-    <row r="10" spans="1:20" ht="30">
+      <c r="R9" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S9" s="21"/>
+      <c r="T9" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" ht="31.5">
       <c r="A10" s="9">
         <v>9</v>
       </c>
@@ -1430,20 +1433,18 @@
         <v>19</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="D10" s="8">
         <v>23</v>
       </c>
       <c r="E10" s="8">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F10" s="8">
         <v>5</v>
       </c>
-      <c r="G10" s="8">
-        <v>2</v>
-      </c>
+      <c r="G10" s="8"/>
       <c r="H10" s="8">
         <v>5</v>
       </c>
@@ -1451,7 +1452,7 @@
         <v>5</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K10" s="10">
         <v>45993</v>
@@ -1460,28 +1461,26 @@
         <v>46055</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O10" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O10" s="26"/>
       <c r="P10" s="34"/>
       <c r="Q10" s="12" t="str">
         <f>HYPERLINK("#'Region Master'!A1","Region Master")</f>
         <v>Region Master</v>
       </c>
       <c r="R10" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S10" s="21"/>
       <c r="T10" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" ht="30">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" ht="31.5">
       <c r="A11" s="44">
         <v>10</v>
       </c>
@@ -1489,26 +1488,24 @@
         <v>19</v>
       </c>
       <c r="C11" s="45" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="D11" s="45">
         <v>26</v>
       </c>
       <c r="E11" s="45">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F11" s="45">
         <v>9</v>
       </c>
-      <c r="G11" s="45">
-        <v>2</v>
-      </c>
+      <c r="G11" s="45"/>
       <c r="H11" s="45">
         <v>9</v>
       </c>
       <c r="I11" s="44"/>
       <c r="J11" s="46" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K11" s="46">
         <v>45994</v>
@@ -1516,23 +1513,21 @@
       <c r="L11" s="49"/>
       <c r="M11" s="49"/>
       <c r="N11" s="46" t="s">
-        <v>23</v>
-      </c>
-      <c r="O11" s="47" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O11" s="47"/>
       <c r="P11" s="49"/>
       <c r="Q11" s="48" t="str">
         <f>HYPERLINK("#'FF Port Master'!A1","FF Port Master")</f>
         <v>FF Port Master</v>
       </c>
       <c r="R11" s="46" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S11" s="49"/>
       <c r="T11" s="23"/>
     </row>
-    <row r="12" spans="1:20" ht="30">
+    <row r="12" spans="1:20" ht="31.5">
       <c r="A12" s="22">
         <v>11</v>
       </c>
@@ -1540,26 +1535,24 @@
         <v>19</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="D12" s="13">
         <v>19</v>
       </c>
       <c r="E12" s="13">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F12" s="13">
         <v>8</v>
       </c>
-      <c r="G12" s="13">
-        <v>2</v>
-      </c>
+      <c r="G12" s="13"/>
       <c r="H12" s="13">
         <v>8</v>
       </c>
       <c r="I12" s="24"/>
       <c r="J12" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K12" s="14">
         <v>45995</v>
@@ -1567,23 +1560,21 @@
       <c r="L12" s="23"/>
       <c r="M12" s="23"/>
       <c r="N12" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O12" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O12" s="7"/>
       <c r="P12" s="23"/>
       <c r="Q12" s="6" t="str">
         <f>HYPERLINK("#'Action Master'!A1","Action Master")</f>
         <v>Action Master</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S12" s="23"/>
       <c r="T12" s="23"/>
     </row>
-    <row r="13" spans="1:20" ht="30">
+    <row r="13" spans="1:20" ht="31.5">
       <c r="A13" s="22">
         <v>12</v>
       </c>
@@ -1591,26 +1582,24 @@
         <v>19</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="D13" s="13">
         <v>16</v>
       </c>
       <c r="E13" s="13">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F13" s="13">
         <v>6</v>
       </c>
-      <c r="G13" s="13">
-        <v>2</v>
-      </c>
+      <c r="G13" s="13"/>
       <c r="H13" s="13">
         <v>6</v>
       </c>
       <c r="I13" s="24"/>
       <c r="J13" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K13" s="14">
         <v>46000</v>
@@ -1618,127 +1607,131 @@
       <c r="L13" s="23"/>
       <c r="M13" s="23"/>
       <c r="N13" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O13" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O13" s="7"/>
       <c r="P13" s="23"/>
       <c r="Q13" s="6" t="str">
         <f>HYPERLINK("#'Period Master'!A1","Period Master")</f>
         <v>Period Master</v>
       </c>
       <c r="R13" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S13" s="23"/>
       <c r="T13" s="23"/>
     </row>
     <row r="14" spans="1:20" ht="31.5">
-      <c r="A14" s="44">
+      <c r="A14" s="20">
         <v>13</v>
       </c>
-      <c r="B14" s="45" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="45">
+      <c r="B14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="8">
         <v>18</v>
       </c>
-      <c r="E14" s="45">
-        <v>10</v>
-      </c>
-      <c r="F14" s="45">
+      <c r="E14" s="8">
+        <v>12</v>
+      </c>
+      <c r="F14" s="8">
         <v>6</v>
       </c>
-      <c r="G14" s="45">
-        <v>2</v>
-      </c>
-      <c r="H14" s="45">
+      <c r="G14" s="8"/>
+      <c r="H14" s="8">
         <v>6</v>
       </c>
-      <c r="I14" s="44"/>
-      <c r="J14" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="K14" s="46">
+      <c r="I14" s="8">
+        <v>6</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K14" s="10">
         <v>46000</v>
       </c>
-      <c r="L14" s="49"/>
-      <c r="M14" s="49"/>
-      <c r="N14" s="46" t="s">
-        <v>79</v>
-      </c>
-      <c r="O14" s="47" t="s">
+      <c r="L14" s="10">
+        <v>46079</v>
+      </c>
+      <c r="M14" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="P14" s="49"/>
-      <c r="Q14" s="48" t="str">
+      <c r="N14" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O14" s="26"/>
+      <c r="P14" s="21"/>
+      <c r="Q14" s="12" t="str">
         <f>HYPERLINK("#'Cost Center Master'!A1","Cost Center Master")</f>
         <v>Cost Center Master</v>
       </c>
-      <c r="R14" s="46" t="s">
+      <c r="R14" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S14" s="21"/>
+      <c r="T14" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" ht="31.5">
+      <c r="A15" s="20">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="8">
+        <v>18</v>
+      </c>
+      <c r="E15" s="8">
+        <v>12</v>
+      </c>
+      <c r="F15" s="8">
+        <v>6</v>
+      </c>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8">
+        <v>6</v>
+      </c>
+      <c r="I15" s="8">
+        <v>6</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" s="10">
+        <v>46001</v>
+      </c>
+      <c r="L15" s="10">
+        <v>46079</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N15" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="S14" s="49"/>
-      <c r="T14" s="23"/>
-    </row>
-    <row r="15" spans="1:20" ht="30">
-      <c r="A15" s="44">
-        <v>14</v>
-      </c>
-      <c r="B15" s="45" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" s="45">
-        <v>18</v>
-      </c>
-      <c r="E15" s="45">
-        <v>10</v>
-      </c>
-      <c r="F15" s="45">
-        <v>6</v>
-      </c>
-      <c r="G15" s="45">
-        <v>2</v>
-      </c>
-      <c r="H15" s="45">
-        <v>6</v>
-      </c>
-      <c r="I15" s="45">
-        <v>6</v>
-      </c>
-      <c r="J15" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="K15" s="46">
-        <v>46001</v>
-      </c>
-      <c r="L15" s="49"/>
-      <c r="M15" s="49"/>
-      <c r="N15" s="46" t="s">
-        <v>23</v>
-      </c>
-      <c r="O15" s="47" t="s">
-        <v>24</v>
-      </c>
-      <c r="P15" s="49"/>
-      <c r="Q15" s="48" t="str">
+      <c r="O15" s="26"/>
+      <c r="P15" s="21"/>
+      <c r="Q15" s="12" t="str">
         <f>HYPERLINK("#'IMO Master'!A1","IMO Master")</f>
         <v>IMO Master</v>
       </c>
-      <c r="R15" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="S15" s="49"/>
-      <c r="T15" s="23"/>
-    </row>
-    <row r="16" spans="1:20" ht="30">
+      <c r="R15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S15" s="21"/>
+      <c r="T15" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" ht="31.5">
       <c r="A16" s="9">
         <v>15</v>
       </c>
@@ -1746,20 +1739,18 @@
         <v>19</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="D16" s="8">
         <v>15</v>
       </c>
       <c r="E16" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F16" s="8">
         <v>6</v>
       </c>
-      <c r="G16" s="8">
-        <v>2</v>
-      </c>
+      <c r="G16" s="8"/>
       <c r="H16" s="8">
         <v>6</v>
       </c>
@@ -1767,7 +1758,7 @@
         <v>6</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K16" s="10">
         <v>46001</v>
@@ -1775,27 +1766,27 @@
       <c r="L16" s="10">
         <v>46055</v>
       </c>
-      <c r="M16" s="21"/>
+      <c r="M16" s="10" t="s">
+        <v>24</v>
+      </c>
       <c r="N16" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O16" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O16" s="26"/>
       <c r="P16" s="21"/>
       <c r="Q16" s="12" t="str">
         <f>HYPERLINK("#'Unit Master'!A1","Unit Master")</f>
         <v>Unit Master</v>
       </c>
       <c r="R16" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S16" s="21"/>
       <c r="T16" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" ht="30">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" ht="31.5">
       <c r="A17" s="20">
         <v>16</v>
       </c>
@@ -1803,20 +1794,18 @@
         <v>19</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="D17" s="8">
         <v>23</v>
       </c>
       <c r="E17" s="8">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F17" s="8">
         <v>6</v>
       </c>
-      <c r="G17" s="8">
-        <v>2</v>
-      </c>
+      <c r="G17" s="8"/>
       <c r="H17" s="8">
         <v>6</v>
       </c>
@@ -1824,7 +1813,7 @@
         <v>6</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K17" s="10">
         <v>46002</v>
@@ -1832,24 +1821,24 @@
       <c r="L17" s="10">
         <v>46063</v>
       </c>
-      <c r="M17" s="21"/>
+      <c r="M17" s="10" t="s">
+        <v>24</v>
+      </c>
       <c r="N17" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="O17" s="26" t="s">
-        <v>24</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="O17" s="26"/>
       <c r="P17" s="21"/>
       <c r="Q17" s="12" t="str">
         <f>HYPERLINK("#'CHA Service'!A1","CHA Service")</f>
         <v>CHA Service</v>
       </c>
       <c r="R17" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S17" s="21"/>
       <c r="T17" s="7" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:20" ht="31.5">
@@ -1860,7 +1849,7 @@
         <v>19</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="D18" s="15">
         <v>60</v>
@@ -1879,7 +1868,7 @@
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K18" s="4">
         <v>46003</v>
@@ -1887,7 +1876,7 @@
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
       <c r="N18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O18" s="7"/>
       <c r="P18" s="5"/>
@@ -1896,7 +1885,7 @@
         <v>Pricing</v>
       </c>
       <c r="R18" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S18" s="5"/>
       <c r="T18" s="23"/>
@@ -1909,7 +1898,7 @@
         <v>19</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="D19" s="36">
         <v>59</v>
@@ -1928,7 +1917,7 @@
       </c>
       <c r="I19" s="22"/>
       <c r="J19" s="37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K19" s="37">
         <v>46007</v>
@@ -1936,7 +1925,7 @@
       <c r="L19" s="38"/>
       <c r="M19" s="38"/>
       <c r="N19" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O19" s="25"/>
       <c r="P19" s="38"/>
@@ -1945,110 +1934,120 @@
         <v>Sea Charge Master</v>
       </c>
       <c r="R19" s="37" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S19" s="37"/>
       <c r="T19" s="23"/>
     </row>
     <row r="20" spans="1:20" ht="31.5">
-      <c r="A20" s="22">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="13">
+      <c r="A20" s="20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="8">
         <v>30</v>
       </c>
-      <c r="E20" s="2">
-        <v>19</v>
-      </c>
-      <c r="F20" s="13">
+      <c r="E20" s="8">
+        <v>23</v>
+      </c>
+      <c r="F20" s="8">
         <v>7</v>
       </c>
-      <c r="G20" s="13">
-        <v>4</v>
-      </c>
-      <c r="H20" s="2">
+      <c r="G20" s="8"/>
+      <c r="H20" s="8">
         <v>7</v>
       </c>
-      <c r="I20" s="22"/>
-      <c r="J20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="K20" s="4">
+      <c r="I20" s="8">
+        <v>7</v>
+      </c>
+      <c r="J20" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K20" s="10">
         <v>46011</v>
       </c>
-      <c r="L20" s="23"/>
-      <c r="M20" s="23"/>
-      <c r="N20" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O20" s="25"/>
-      <c r="P20" s="23"/>
-      <c r="Q20" s="6" t="str">
+      <c r="L20" s="10">
+        <v>46079</v>
+      </c>
+      <c r="M20" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N20" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O20" s="43"/>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="12" t="str">
         <f>HYPERLINK("#'Segment Master'!A1","Segment Master")</f>
         <v>Segment Master</v>
       </c>
-      <c r="R20" s="4" t="s">
+      <c r="R20" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S20" s="21"/>
+      <c r="T20" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" ht="31.5">
+      <c r="A21" s="20">
+        <v>20</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="8">
         <v>25</v>
       </c>
-      <c r="S20" s="23"/>
-      <c r="T20" s="23"/>
-    </row>
-    <row r="21" spans="1:20" ht="30">
-      <c r="A21" s="22">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="13">
+      <c r="E21" s="8">
+        <v>17</v>
+      </c>
+      <c r="F21" s="8">
+        <v>8</v>
+      </c>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8">
+        <v>8</v>
+      </c>
+      <c r="I21" s="8">
+        <v>8</v>
+      </c>
+      <c r="J21" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K21" s="10">
+        <v>46011</v>
+      </c>
+      <c r="L21" s="10">
+        <v>46079</v>
+      </c>
+      <c r="M21" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N21" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="2">
-        <v>15</v>
-      </c>
-      <c r="F21" s="13">
-        <v>8</v>
-      </c>
-      <c r="G21" s="13">
-        <v>2</v>
-      </c>
-      <c r="H21" s="2">
-        <v>8</v>
-      </c>
-      <c r="I21" s="22"/>
-      <c r="J21" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="K21" s="4">
-        <v>46011</v>
-      </c>
-      <c r="L21" s="23"/>
-      <c r="M21" s="23"/>
-      <c r="N21" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O21" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="P21" s="23"/>
-      <c r="Q21" s="6" t="str">
+      <c r="O21" s="26"/>
+      <c r="P21" s="21"/>
+      <c r="Q21" s="12" t="str">
         <f>HYPERLINK("#'Trigger Master'!A1","Trigger Master")</f>
         <v>Trigger Master</v>
       </c>
-      <c r="R21" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="S21" s="23"/>
-      <c r="T21" s="23"/>
+      <c r="R21" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S21" s="21"/>
+      <c r="T21" s="7" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="22" spans="1:20" ht="31.5">
       <c r="A22" s="22">
@@ -2058,26 +2057,24 @@
         <v>19</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="D22" s="13">
         <v>15</v>
       </c>
       <c r="E22" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F22" s="13">
         <v>5</v>
       </c>
-      <c r="G22" s="13">
-        <v>2</v>
-      </c>
+      <c r="G22" s="13"/>
       <c r="H22" s="2">
         <v>5</v>
       </c>
       <c r="I22" s="22"/>
       <c r="J22" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K22" s="4">
         <v>46013</v>
@@ -2085,23 +2082,21 @@
       <c r="L22" s="23"/>
       <c r="M22" s="23"/>
       <c r="N22" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O22" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O22" s="7"/>
       <c r="P22" s="23"/>
       <c r="Q22" s="6" t="str">
         <f>HYPERLINK("#'Principle Line HBL Master'!A1","Principle Line HBL Master")</f>
         <v>Principle Line HBL Master</v>
       </c>
       <c r="R22" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S22" s="23"/>
       <c r="T22" s="23"/>
     </row>
-    <row r="23" spans="1:20" ht="30">
+    <row r="23" spans="1:20" ht="31.5">
       <c r="A23" s="22">
         <v>22</v>
       </c>
@@ -2109,26 +2104,24 @@
         <v>19</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D23" s="13">
         <v>19</v>
       </c>
       <c r="E23" s="2">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F23" s="13">
         <v>6</v>
       </c>
-      <c r="G23" s="13">
-        <v>2</v>
-      </c>
+      <c r="G23" s="13"/>
       <c r="H23" s="2">
         <v>6</v>
       </c>
       <c r="I23" s="22"/>
       <c r="J23" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K23" s="4">
         <v>46014</v>
@@ -2136,18 +2129,16 @@
       <c r="L23" s="23"/>
       <c r="M23" s="23"/>
       <c r="N23" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O23" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O23" s="7"/>
       <c r="P23" s="23"/>
       <c r="Q23" s="6" t="str">
         <f>HYPERLINK("#'Project Type Master'!A1","Project Type Master")</f>
         <v>Project Type Master</v>
       </c>
       <c r="R23" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S23" s="23"/>
       <c r="T23" s="23"/>
@@ -2160,26 +2151,24 @@
         <v>19</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="D24" s="13">
         <v>23</v>
       </c>
       <c r="E24" s="2">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F24" s="13">
         <v>6</v>
       </c>
-      <c r="G24" s="13">
-        <v>2</v>
-      </c>
+      <c r="G24" s="13"/>
       <c r="H24" s="2">
         <v>6</v>
       </c>
       <c r="I24" s="22"/>
       <c r="J24" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K24" s="4">
         <v>46014</v>
@@ -2187,23 +2176,21 @@
       <c r="L24" s="23"/>
       <c r="M24" s="23"/>
       <c r="N24" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O24" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O24" s="7"/>
       <c r="P24" s="23"/>
       <c r="Q24" s="6" t="str">
         <f>HYPERLINK("#'Notes Master'!A1","Notes Master")</f>
         <v>Notes Master</v>
       </c>
       <c r="R24" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S24" s="23"/>
       <c r="T24" s="23"/>
     </row>
-    <row r="25" spans="1:20" ht="30">
+    <row r="25" spans="1:20" ht="31.5">
       <c r="A25" s="22">
         <v>24</v>
       </c>
@@ -2211,26 +2198,24 @@
         <v>19</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="D25" s="13">
         <v>19</v>
       </c>
       <c r="E25" s="2">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F25" s="13">
         <v>6</v>
       </c>
-      <c r="G25" s="13">
-        <v>2</v>
-      </c>
+      <c r="G25" s="13"/>
       <c r="H25" s="2">
         <v>6</v>
       </c>
       <c r="I25" s="22"/>
       <c r="J25" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K25" s="4">
         <v>46015</v>
@@ -2238,23 +2223,21 @@
       <c r="L25" s="23"/>
       <c r="M25" s="23"/>
       <c r="N25" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O25" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O25" s="7"/>
       <c r="P25" s="23"/>
       <c r="Q25" s="6" t="str">
         <f>HYPERLINK("#'Vessel'!A1","Vessel")</f>
         <v>Vessel</v>
       </c>
       <c r="R25" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S25" s="23"/>
       <c r="T25" s="23"/>
     </row>
-    <row r="26" spans="1:20" ht="30">
+    <row r="26" spans="1:20" ht="31.5">
       <c r="A26" s="22">
         <v>25</v>
       </c>
@@ -2262,26 +2245,24 @@
         <v>19</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="D26" s="13">
         <v>76</v>
       </c>
       <c r="E26" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F26" s="13">
         <v>27</v>
       </c>
-      <c r="G26" s="13">
-        <v>2</v>
-      </c>
+      <c r="G26" s="13"/>
       <c r="H26" s="15">
         <v>18</v>
       </c>
       <c r="I26" s="22"/>
       <c r="J26" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K26" s="4">
         <v>46017</v>
@@ -2289,18 +2270,16 @@
       <c r="L26" s="23"/>
       <c r="M26" s="23"/>
       <c r="N26" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>24</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="O26" s="1"/>
       <c r="P26" s="23"/>
       <c r="Q26" s="6" t="str">
         <f>HYPERLINK("#'Schedule'!A1","Schedule")</f>
         <v>Schedule</v>
       </c>
       <c r="R26" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S26" s="23"/>
       <c r="T26" s="23"/>
@@ -2313,7 +2292,7 @@
         <v>19</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="D27" s="13">
         <v>20</v>
@@ -2330,7 +2309,7 @@
       </c>
       <c r="I27" s="23"/>
       <c r="J27" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K27" s="4">
         <v>46023</v>
@@ -2338,7 +2317,7 @@
       <c r="L27" s="23"/>
       <c r="M27" s="23"/>
       <c r="N27" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O27" s="1"/>
       <c r="P27" s="23"/>
@@ -2347,7 +2326,7 @@
         <v>Shipment Status</v>
       </c>
       <c r="R27" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S27" s="23"/>
       <c r="T27" s="23"/>
@@ -2360,7 +2339,7 @@
         <v>19</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="D28" s="13">
         <v>16</v>
@@ -2377,7 +2356,7 @@
       </c>
       <c r="I28" s="23"/>
       <c r="J28" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K28" s="4">
         <v>46027</v>
@@ -2385,7 +2364,7 @@
       <c r="L28" s="23"/>
       <c r="M28" s="23"/>
       <c r="N28" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O28" s="25"/>
       <c r="P28" s="23"/>
@@ -2394,7 +2373,7 @@
         <v>Destuffing</v>
       </c>
       <c r="R28" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S28" s="23"/>
       <c r="T28" s="23"/>
@@ -2407,7 +2386,7 @@
         <v>19</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="D29" s="13">
         <v>15</v>
@@ -2424,7 +2403,7 @@
       </c>
       <c r="I29" s="23"/>
       <c r="J29" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K29" s="4">
         <v>46027</v>
@@ -2432,7 +2411,7 @@
       <c r="L29" s="23"/>
       <c r="M29" s="23"/>
       <c r="N29" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O29" s="25"/>
       <c r="P29" s="23"/>
@@ -2441,7 +2420,7 @@
         <v>Document</v>
       </c>
       <c r="R29" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S29" s="23"/>
       <c r="T29" s="23"/>
@@ -2454,7 +2433,7 @@
         <v>19</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="D30" s="13">
         <v>21</v>
@@ -2471,7 +2450,7 @@
       </c>
       <c r="I30" s="23"/>
       <c r="J30" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K30" s="4">
         <v>46028</v>
@@ -2486,7 +2465,7 @@
         <v>Container</v>
       </c>
       <c r="R30" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S30" s="23"/>
       <c r="T30" s="23"/>
@@ -2499,7 +2478,7 @@
         <v>19</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="D31" s="8">
         <v>16</v>
@@ -2518,7 +2497,7 @@
         <v>9</v>
       </c>
       <c r="J31" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K31" s="10">
         <v>46030</v>
@@ -2526,9 +2505,11 @@
       <c r="L31" s="10">
         <v>46063</v>
       </c>
-      <c r="M31" s="21"/>
+      <c r="M31" s="10" t="s">
+        <v>24</v>
+      </c>
       <c r="N31" s="10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="O31" s="43"/>
       <c r="P31" s="21"/>
@@ -2537,11 +2518,11 @@
         <v>Stuffing Master</v>
       </c>
       <c r="R31" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S31" s="21"/>
       <c r="T31" s="25" t="s">
-        <v>83</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="31.5">
@@ -2552,7 +2533,7 @@
         <v>19</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="D32" s="13">
         <v>13</v>
@@ -2569,7 +2550,7 @@
       </c>
       <c r="I32" s="23"/>
       <c r="J32" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K32" s="4">
         <v>46029</v>
@@ -2577,7 +2558,7 @@
       <c r="L32" s="23"/>
       <c r="M32" s="23"/>
       <c r="N32" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O32" s="25"/>
       <c r="P32" s="23"/>
@@ -2586,7 +2567,7 @@
         <v>Daily Currency Rate</v>
       </c>
       <c r="R32" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S32" s="23"/>
       <c r="T32" s="23"/>
@@ -2599,7 +2580,7 @@
         <v>19</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="D33" s="13">
         <v>18</v>
@@ -2616,7 +2597,7 @@
       </c>
       <c r="I33" s="23"/>
       <c r="J33" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K33" s="4">
         <v>46030</v>
@@ -2624,7 +2605,7 @@
       <c r="L33" s="23"/>
       <c r="M33" s="23"/>
       <c r="N33" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O33" s="25"/>
       <c r="P33" s="23"/>
@@ -2633,7 +2614,7 @@
         <v>Container Yard Master</v>
       </c>
       <c r="R33" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S33" s="23"/>
       <c r="T33" s="23"/>
@@ -2646,7 +2627,7 @@
         <v>19</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="D34" s="13">
         <v>38</v>
@@ -2665,7 +2646,7 @@
       </c>
       <c r="I34" s="23"/>
       <c r="J34" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K34" s="4">
         <v>46036</v>
@@ -2673,7 +2654,7 @@
       <c r="L34" s="23"/>
       <c r="M34" s="23"/>
       <c r="N34" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O34" s="25"/>
       <c r="P34" s="23"/>
@@ -2682,7 +2663,7 @@
         <v>Create Branch</v>
       </c>
       <c r="R34" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S34" s="23"/>
       <c r="T34" s="23"/>
@@ -2695,7 +2676,7 @@
         <v>19</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="D35" s="13">
         <v>14</v>
@@ -2712,24 +2693,24 @@
       </c>
       <c r="I35" s="23"/>
       <c r="J35" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K35" s="4">
-        <v>46037</v>
+        <v>46080</v>
       </c>
       <c r="L35" s="23"/>
       <c r="M35" s="23"/>
       <c r="N35" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O35" s="25"/>
       <c r="P35" s="23"/>
       <c r="Q35" s="6" t="str">
-        <f>HYPERLINK("#'Activity'!A1","Activity")</f>
-        <v>Activity</v>
+        <f>HYPERLINK("#'Shipment Plan Master'!A1","Shipment Plan Master")</f>
+        <v>Shipment Plan Master</v>
       </c>
       <c r="R35" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S35" s="23"/>
       <c r="T35" s="23"/>
@@ -2739,10 +2720,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="30" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="C36" s="30" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D36" s="30">
         <v>115</v>
@@ -2753,7 +2734,7 @@
       <c r="H36" s="31"/>
       <c r="I36" s="31"/>
       <c r="J36" s="32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K36" s="32">
         <v>46041</v>
@@ -2761,7 +2742,7 @@
       <c r="L36" s="31"/>
       <c r="M36" s="31"/>
       <c r="N36" s="32" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O36" s="33"/>
       <c r="P36" s="31"/>
@@ -2770,7 +2751,7 @@
         <v>Shipment Reg-Shipment</v>
       </c>
       <c r="R36" s="32" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S36" s="31"/>
       <c r="T36" s="23"/>
@@ -2783,7 +2764,7 @@
         <v>19</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="D37" s="13">
         <v>15</v>
@@ -2794,7 +2775,7 @@
       <c r="H37" s="13"/>
       <c r="I37" s="13"/>
       <c r="J37" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K37" s="14">
         <v>46052</v>
@@ -2802,7 +2783,7 @@
       <c r="L37" s="27"/>
       <c r="M37" s="27"/>
       <c r="N37" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O37" s="28"/>
       <c r="P37" s="41"/>
@@ -2811,7 +2792,7 @@
         <v>CHA Port Master</v>
       </c>
       <c r="R37" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S37" s="27"/>
       <c r="T37" s="23"/>
@@ -2824,7 +2805,7 @@
         <v>19</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="D38" s="13">
         <v>15</v>
@@ -2835,7 +2816,7 @@
       <c r="H38" s="13"/>
       <c r="I38" s="13"/>
       <c r="J38" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K38" s="14">
         <v>46053</v>
@@ -2843,7 +2824,7 @@
       <c r="L38" s="27"/>
       <c r="M38" s="27"/>
       <c r="N38" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O38" s="28"/>
       <c r="P38" s="41"/>
@@ -2852,7 +2833,7 @@
         <v>Transporter Master</v>
       </c>
       <c r="R38" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S38" s="27"/>
       <c r="T38" s="23"/>
@@ -2865,7 +2846,7 @@
         <v>19</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="D39" s="13">
         <v>25</v>
@@ -2876,7 +2857,7 @@
       <c r="H39" s="13"/>
       <c r="I39" s="13"/>
       <c r="J39" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K39" s="14">
         <v>46055</v>
@@ -2884,7 +2865,7 @@
       <c r="L39" s="27"/>
       <c r="M39" s="27"/>
       <c r="N39" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O39" s="28"/>
       <c r="P39" s="41"/>
@@ -2893,7 +2874,7 @@
         <v>Drawback Schedule</v>
       </c>
       <c r="R39" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S39" s="27"/>
       <c r="T39" s="23"/>
@@ -2906,7 +2887,7 @@
         <v>19</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="D40" s="13">
         <v>14</v>
@@ -2917,7 +2898,7 @@
       <c r="H40" s="13"/>
       <c r="I40" s="13"/>
       <c r="J40" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K40" s="14">
         <v>46057</v>
@@ -2925,7 +2906,7 @@
       <c r="L40" s="27"/>
       <c r="M40" s="27"/>
       <c r="N40" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O40" s="28"/>
       <c r="P40" s="41"/>
@@ -2934,7 +2915,7 @@
         <v>EDI-Country</v>
       </c>
       <c r="R40" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S40" s="27"/>
       <c r="T40" s="23"/>
@@ -2947,7 +2928,7 @@
         <v>19</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="D41" s="13">
         <v>5</v>
@@ -2958,7 +2939,7 @@
       <c r="H41" s="13"/>
       <c r="I41" s="13"/>
       <c r="J41" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K41" s="14">
         <v>46057</v>
@@ -2966,7 +2947,7 @@
       <c r="L41" s="27"/>
       <c r="M41" s="27"/>
       <c r="N41" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O41" s="28"/>
       <c r="P41" s="41"/>
@@ -2975,7 +2956,7 @@
         <v>Licence Master New</v>
       </c>
       <c r="R41" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S41" s="27"/>
       <c r="T41" s="23"/>
@@ -2988,7 +2969,7 @@
         <v>19</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="D42" s="13">
         <v>17</v>
@@ -2999,7 +2980,7 @@
       <c r="H42" s="13"/>
       <c r="I42" s="13"/>
       <c r="J42" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K42" s="14">
         <v>46058</v>
@@ -3007,7 +2988,7 @@
       <c r="L42" s="27"/>
       <c r="M42" s="27"/>
       <c r="N42" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O42" s="28"/>
       <c r="P42" s="41"/>
@@ -3016,7 +2997,7 @@
         <v>eSanchit Code</v>
       </c>
       <c r="R42" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S42" s="27"/>
       <c r="T42" s="23"/>
@@ -3029,7 +3010,7 @@
         <v>19</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="D43" s="13">
         <v>25</v>
@@ -3040,7 +3021,7 @@
       <c r="H43" s="13"/>
       <c r="I43" s="13"/>
       <c r="J43" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K43" s="14">
         <v>46059</v>
@@ -3048,7 +3029,7 @@
       <c r="L43" s="27"/>
       <c r="M43" s="27"/>
       <c r="N43" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O43" s="28"/>
       <c r="P43" s="41"/>
@@ -3057,7 +3038,7 @@
         <v>CESS Schedule Master</v>
       </c>
       <c r="R43" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S43" s="27"/>
       <c r="T43" s="23"/>
@@ -3070,7 +3051,7 @@
         <v>19</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="D44" s="13">
         <v>19</v>
@@ -3081,7 +3062,7 @@
       <c r="H44" s="13"/>
       <c r="I44" s="13"/>
       <c r="J44" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K44" s="14">
         <v>46060</v>
@@ -3089,7 +3070,7 @@
       <c r="L44" s="27"/>
       <c r="M44" s="27"/>
       <c r="N44" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O44" s="28"/>
       <c r="P44" s="41"/>
@@ -3098,7 +3079,7 @@
         <v>Rodtep Master</v>
       </c>
       <c r="R44" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S44" s="27"/>
       <c r="T44" s="23"/>
@@ -3111,18 +3092,18 @@
         <v>19</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="D45" s="13">
         <v>20</v>
       </c>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="13"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
       <c r="H45" s="13"/>
       <c r="I45" s="13"/>
       <c r="J45" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K45" s="14">
         <v>46062</v>
@@ -3130,7 +3111,7 @@
       <c r="L45" s="27"/>
       <c r="M45" s="27"/>
       <c r="N45" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O45" s="28"/>
       <c r="P45" s="41"/>
@@ -3139,7 +3120,7 @@
         <v>Vehicle Owner Master</v>
       </c>
       <c r="R45" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S45" s="27"/>
       <c r="T45" s="23"/>
@@ -3152,7 +3133,7 @@
         <v>19</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="D46" s="13">
         <v>26</v>
@@ -3163,7 +3144,7 @@
       <c r="H46" s="23"/>
       <c r="I46" s="23"/>
       <c r="J46" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K46" s="14">
         <v>46063</v>
@@ -3171,7 +3152,7 @@
       <c r="L46" s="23"/>
       <c r="M46" s="23"/>
       <c r="N46" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O46" s="25"/>
       <c r="P46" s="23"/>
@@ -3180,7 +3161,7 @@
         <v>Item Template Master</v>
       </c>
       <c r="R46" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="S46" s="23"/>
     </row>
@@ -3192,7 +3173,7 @@
         <v>19</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="D47" s="13">
         <v>26</v>
@@ -3203,7 +3184,7 @@
       <c r="H47" s="23"/>
       <c r="I47" s="23"/>
       <c r="J47" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K47" s="14">
         <v>46064</v>
@@ -3211,7 +3192,7 @@
       <c r="L47" s="23"/>
       <c r="M47" s="23"/>
       <c r="N47" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O47" s="25"/>
       <c r="P47" s="23"/>
@@ -3220,7 +3201,7 @@
         <v>ROSL DBK</v>
       </c>
       <c r="R47" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48" spans="1:20" ht="31.5">
@@ -3231,7 +3212,7 @@
         <v>19</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="D48" s="13">
         <v>29</v>
@@ -3242,7 +3223,7 @@
       <c r="H48" s="23"/>
       <c r="I48" s="23"/>
       <c r="J48" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K48" s="14">
         <v>46066</v>
@@ -3250,7 +3231,7 @@
       <c r="L48" s="23"/>
       <c r="M48" s="23"/>
       <c r="N48" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O48" s="25"/>
       <c r="P48" s="23"/>
@@ -3259,7 +3240,7 @@
         <v>Licence Master</v>
       </c>
       <c r="R48" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="49" spans="1:18" ht="31.5">
@@ -3267,13 +3248,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C49" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C49" s="13" t="s">
-        <v>86</v>
-      </c>
       <c r="D49" s="13">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="E49" s="27"/>
       <c r="F49" s="27"/>
@@ -3281,7 +3262,7 @@
       <c r="H49" s="27"/>
       <c r="I49" s="27"/>
       <c r="J49" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K49" s="14">
         <v>46069</v>
@@ -3289,7 +3270,7 @@
       <c r="L49" s="27"/>
       <c r="M49" s="27"/>
       <c r="N49" s="14" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="O49" s="51"/>
       <c r="P49" s="27"/>
@@ -3298,7 +3279,163 @@
         <v>Ledger Account</v>
       </c>
       <c r="R49" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" ht="31.5">
+      <c r="A50" s="24">
+        <v>49</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D50" s="13">
+        <v>45</v>
+      </c>
+      <c r="E50" s="27"/>
+      <c r="F50" s="27"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="27"/>
+      <c r="I50" s="27"/>
+      <c r="J50" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K50" s="14">
+        <v>46078</v>
+      </c>
+      <c r="L50" s="27"/>
+      <c r="M50" s="27"/>
+      <c r="N50" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O50" s="51"/>
+      <c r="P50" s="27"/>
+      <c r="Q50" s="6" t="str">
+        <f>HYPERLINK("#'GST Charges'!A1","GST Charges")</f>
+        <v>GST Charges</v>
+      </c>
+      <c r="R50" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" ht="31.5">
+      <c r="A51" s="24">
+        <v>50</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D51" s="2">
+        <v>11</v>
+      </c>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K51" s="14">
+        <v>46080</v>
+      </c>
+      <c r="L51" s="23"/>
+      <c r="M51" s="23"/>
+      <c r="N51" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O51" s="7"/>
+      <c r="P51" s="3"/>
+      <c r="Q51" s="6" t="str">
+        <f>HYPERLINK("#'Shipment Plan'!A1","Shipment Plan")</f>
+        <v>Shipment Plan</v>
+      </c>
+      <c r="R51" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="31.5">
+      <c r="A52" s="24">
+        <v>51</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D52" s="2">
+        <v>12</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K52" s="14">
+        <v>46084</v>
+      </c>
+      <c r="L52" s="23"/>
+      <c r="M52" s="23"/>
+      <c r="N52" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O52" s="7"/>
+      <c r="P52" s="3"/>
+      <c r="Q52" s="6" t="str">
+        <f>HYPERLINK("#'TDS Schedule'!A1","TDS Schedule")</f>
+        <v>TDS Schedule</v>
+      </c>
+      <c r="R52" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" ht="31.5">
+      <c r="A53" s="24">
+        <v>52</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D53" s="2">
+        <v>5</v>
+      </c>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K53" s="14">
+        <v>46084</v>
+      </c>
+      <c r="L53" s="23"/>
+      <c r="M53" s="23"/>
+      <c r="N53" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O53" s="7"/>
+      <c r="P53" s="3"/>
+      <c r="Q53" s="6" t="str">
+        <f>HYPERLINK("#'Charge Rules'!A1","Charge Rules")</f>
+        <v>Charge Rules</v>
+      </c>
+      <c r="R53" s="14" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -3318,27 +3455,27 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
All test case update on 13-03-2026
</commit_message>
<xml_diff>
--- a/Icaffe_TestCases_Tracker_Log.xlsx
+++ b/Icaffe_TestCases_Tracker_Log.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="330" windowWidth="28455" windowHeight="12255"/>
+    <workbookView xWindow="360" yWindow="330" windowWidth="28455" windowHeight="12255" tabRatio="678"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker Log" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="96">
   <si>
     <t>SL No.</t>
   </si>
@@ -215,10 +215,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Charge Master - Cost/Revenue Master
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">EDI Master --&gt; ROSL DBK
 </t>
   </si>
@@ -230,9 +226,6 @@
 </t>
   </si>
   <si>
-    <t>Working</t>
-  </si>
-  <si>
     <t xml:space="preserve">Party --&gt; Bank BRO
 </t>
   </si>
@@ -333,6 +326,37 @@
   </si>
   <si>
     <t xml:space="preserve">Master -&gt; Charge Rules
+</t>
+  </si>
+  <si>
+    <t>Charge Master - Cost/Revenue Master</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; Item Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; Division Mapping
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; TDS Party
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; SAC Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; Depreciation Rates Master
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master -&gt; Merge Accounts
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voucher -&gt; Receipt Voucher
 </t>
   </si>
 </sst>
@@ -394,7 +418,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -426,13 +450,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -484,7 +502,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -567,6 +585,35 @@
     <xf numFmtId="14" fontId="6" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -577,54 +624,16 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="7" borderId="2" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -921,7 +930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T53"/>
+  <dimension ref="A1:T60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="18"/>
@@ -1005,7 +1014,7 @@
       <c r="S1" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="42" t="s">
+      <c r="T1" s="37" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1017,7 +1026,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D2" s="8">
         <v>55</v>
@@ -1072,7 +1081,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D3" s="8">
         <v>75</v>
@@ -1127,7 +1136,7 @@
         <v>19</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D4" s="8">
         <v>29</v>
@@ -1182,7 +1191,7 @@
         <v>19</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D5" s="8">
         <v>29</v>
@@ -1237,7 +1246,7 @@
         <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2">
         <v>21</v>
@@ -1284,7 +1293,7 @@
         <v>19</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D7" s="2">
         <v>0</v>
@@ -1323,7 +1332,7 @@
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D8" s="8">
         <v>20</v>
@@ -1378,7 +1387,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D9" s="8">
         <v>25</v>
@@ -1433,7 +1442,7 @@
         <v>19</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D10" s="8">
         <v>23</v>
@@ -1467,7 +1476,7 @@
         <v>25</v>
       </c>
       <c r="O10" s="26"/>
-      <c r="P10" s="34"/>
+      <c r="P10" s="30"/>
       <c r="Q10" s="12" t="str">
         <f>HYPERLINK("#'Region Master'!A1","Region Master")</f>
         <v>Region Master</v>
@@ -1481,51 +1490,59 @@
       </c>
     </row>
     <row r="11" spans="1:20" ht="31.5">
-      <c r="A11" s="44">
+      <c r="A11" s="20">
         <v>10</v>
       </c>
-      <c r="B11" s="45" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="45" t="s">
-        <v>73</v>
-      </c>
-      <c r="D11" s="45">
+      <c r="B11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="8">
         <v>26</v>
       </c>
-      <c r="E11" s="45">
+      <c r="E11" s="8">
         <v>17</v>
       </c>
-      <c r="F11" s="45">
+      <c r="F11" s="8">
         <v>9</v>
       </c>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45">
+      <c r="G11" s="8"/>
+      <c r="H11" s="8">
         <v>9</v>
       </c>
-      <c r="I11" s="44"/>
-      <c r="J11" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="K11" s="46">
+      <c r="I11" s="8">
+        <v>9</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" s="10">
         <v>45994</v>
       </c>
-      <c r="L11" s="49"/>
-      <c r="M11" s="49"/>
-      <c r="N11" s="46" t="s">
-        <v>22</v>
-      </c>
-      <c r="O11" s="47"/>
-      <c r="P11" s="49"/>
-      <c r="Q11" s="48" t="str">
+      <c r="L11" s="10">
+        <v>46086</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O11" s="26"/>
+      <c r="P11" s="21"/>
+      <c r="Q11" s="12" t="str">
         <f>HYPERLINK("#'FF Port Master'!A1","FF Port Master")</f>
         <v>FF Port Master</v>
       </c>
-      <c r="R11" s="46" t="s">
-        <v>23</v>
-      </c>
-      <c r="S11" s="49"/>
-      <c r="T11" s="23"/>
+      <c r="R11" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S11" s="21"/>
+      <c r="T11" s="7" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="12" spans="1:20" ht="31.5">
       <c r="A12" s="22">
@@ -1535,7 +1552,7 @@
         <v>19</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D12" s="13">
         <v>19</v>
@@ -1582,7 +1599,7 @@
         <v>19</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D13" s="13">
         <v>16</v>
@@ -1684,7 +1701,7 @@
         <v>19</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D15" s="8">
         <v>18</v>
@@ -1739,7 +1756,7 @@
         <v>19</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D16" s="8">
         <v>15</v>
@@ -1794,7 +1811,7 @@
         <v>19</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D17" s="8">
         <v>23</v>
@@ -1890,53 +1907,53 @@
       <c r="S18" s="5"/>
       <c r="T18" s="23"/>
     </row>
-    <row r="19" spans="1:20" ht="47.25">
+    <row r="19" spans="1:20" ht="31.5">
       <c r="A19" s="22">
         <v>18</v>
       </c>
-      <c r="B19" s="35" t="s">
+      <c r="B19" s="31" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="32">
         <v>59</v>
       </c>
-      <c r="D19" s="36">
-        <v>59</v>
-      </c>
-      <c r="E19" s="35">
+      <c r="E19" s="31">
         <v>33</v>
       </c>
-      <c r="F19" s="36">
-        <v>20</v>
-      </c>
-      <c r="G19" s="36">
+      <c r="F19" s="32">
+        <v>20</v>
+      </c>
+      <c r="G19" s="32">
         <v>6</v>
       </c>
-      <c r="H19" s="35">
+      <c r="H19" s="31">
         <v>20</v>
       </c>
       <c r="I19" s="22"/>
-      <c r="J19" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="K19" s="37">
+      <c r="J19" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="K19" s="33">
         <v>46007</v>
       </c>
-      <c r="L19" s="38"/>
-      <c r="M19" s="38"/>
-      <c r="N19" s="37" t="s">
+      <c r="L19" s="34"/>
+      <c r="M19" s="34"/>
+      <c r="N19" s="33" t="s">
         <v>22</v>
       </c>
       <c r="O19" s="25"/>
-      <c r="P19" s="38"/>
-      <c r="Q19" s="39" t="str">
+      <c r="P19" s="34"/>
+      <c r="Q19" s="35" t="str">
         <f>HYPERLINK("#'Sea Charge Master'!A1","Sea Charge Master")</f>
         <v>Sea Charge Master</v>
       </c>
-      <c r="R19" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="S19" s="37"/>
+      <c r="R19" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="S19" s="33"/>
       <c r="T19" s="23"/>
     </row>
     <row r="20" spans="1:20" ht="31.5">
@@ -1980,7 +1997,7 @@
       <c r="N20" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="O20" s="43"/>
+      <c r="O20" s="38"/>
       <c r="P20" s="21"/>
       <c r="Q20" s="12" t="str">
         <f>HYPERLINK("#'Segment Master'!A1","Segment Master")</f>
@@ -2002,7 +2019,7 @@
         <v>19</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D21" s="8">
         <v>25</v>
@@ -2050,192 +2067,224 @@
       </c>
     </row>
     <row r="22" spans="1:20" ht="31.5">
-      <c r="A22" s="22">
+      <c r="A22" s="20">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="15" t="s">
+      <c r="B22" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="13">
+      <c r="D22" s="8">
         <v>15</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="8">
         <v>10</v>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="8">
         <v>5</v>
       </c>
-      <c r="G22" s="13"/>
-      <c r="H22" s="2">
+      <c r="G22" s="8"/>
+      <c r="H22" s="8">
         <v>5</v>
       </c>
-      <c r="I22" s="22"/>
-      <c r="J22" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K22" s="4">
+      <c r="I22" s="8">
+        <v>5</v>
+      </c>
+      <c r="J22" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K22" s="10">
         <v>46013</v>
       </c>
-      <c r="L22" s="23"/>
-      <c r="M22" s="23"/>
-      <c r="N22" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="O22" s="7"/>
-      <c r="P22" s="23"/>
-      <c r="Q22" s="6" t="str">
+      <c r="L22" s="10">
+        <v>46090</v>
+      </c>
+      <c r="M22" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N22" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O22" s="26"/>
+      <c r="P22" s="21"/>
+      <c r="Q22" s="12" t="str">
         <f>HYPERLINK("#'Principle Line HBL Master'!A1","Principle Line HBL Master")</f>
         <v>Principle Line HBL Master</v>
       </c>
-      <c r="R22" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="S22" s="23"/>
-      <c r="T22" s="23"/>
+      <c r="R22" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S22" s="21"/>
+      <c r="T22" s="7" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="23" spans="1:20" ht="31.5">
-      <c r="A23" s="22">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="D23" s="13">
-        <v>19</v>
-      </c>
-      <c r="E23" s="2">
+      <c r="A23" s="20">
+        <v>22</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D23" s="8">
+        <v>19</v>
+      </c>
+      <c r="E23" s="8">
         <v>13</v>
       </c>
-      <c r="F23" s="13">
+      <c r="F23" s="8">
         <v>6</v>
       </c>
-      <c r="G23" s="13"/>
-      <c r="H23" s="2">
+      <c r="G23" s="8"/>
+      <c r="H23" s="8">
         <v>6</v>
       </c>
-      <c r="I23" s="22"/>
-      <c r="J23" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K23" s="4">
+      <c r="I23" s="8">
+        <v>6</v>
+      </c>
+      <c r="J23" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K23" s="10">
         <v>46014</v>
       </c>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-      <c r="N23" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="O23" s="7"/>
-      <c r="P23" s="23"/>
-      <c r="Q23" s="6" t="str">
+      <c r="L23" s="10">
+        <v>46090</v>
+      </c>
+      <c r="M23" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N23" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O23" s="26"/>
+      <c r="P23" s="21"/>
+      <c r="Q23" s="12" t="str">
         <f>HYPERLINK("#'Project Type Master'!A1","Project Type Master")</f>
         <v>Project Type Master</v>
       </c>
-      <c r="R23" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="S23" s="23"/>
-      <c r="T23" s="23"/>
+      <c r="R23" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S23" s="21"/>
+      <c r="T23" s="7" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="24" spans="1:20" ht="31.5">
-      <c r="A24" s="22">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C24" s="15" t="s">
+      <c r="A24" s="20">
+        <v>23</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="13">
-        <v>23</v>
-      </c>
-      <c r="E24" s="2">
+      <c r="D24" s="8">
+        <v>23</v>
+      </c>
+      <c r="E24" s="8">
         <v>17</v>
       </c>
-      <c r="F24" s="13">
+      <c r="F24" s="8">
         <v>6</v>
       </c>
-      <c r="G24" s="13"/>
-      <c r="H24" s="2">
+      <c r="G24" s="8"/>
+      <c r="H24" s="8">
         <v>6</v>
       </c>
-      <c r="I24" s="22"/>
-      <c r="J24" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K24" s="4">
+      <c r="I24" s="8">
+        <v>6</v>
+      </c>
+      <c r="J24" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K24" s="10">
         <v>46014</v>
       </c>
-      <c r="L24" s="23"/>
-      <c r="M24" s="23"/>
-      <c r="N24" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="O24" s="7"/>
-      <c r="P24" s="23"/>
-      <c r="Q24" s="6" t="str">
+      <c r="L24" s="10">
+        <v>46090</v>
+      </c>
+      <c r="M24" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N24" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O24" s="26"/>
+      <c r="P24" s="21"/>
+      <c r="Q24" s="12" t="str">
         <f>HYPERLINK("#'Notes Master'!A1","Notes Master")</f>
         <v>Notes Master</v>
       </c>
-      <c r="R24" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="S24" s="23"/>
-      <c r="T24" s="23"/>
+      <c r="R24" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S24" s="21"/>
+      <c r="T24" s="7" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="25" spans="1:20" ht="31.5">
-      <c r="A25" s="22">
+      <c r="A25" s="20">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="D25" s="13">
-        <v>19</v>
-      </c>
-      <c r="E25" s="2">
+      <c r="B25" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="8">
+        <v>19</v>
+      </c>
+      <c r="E25" s="8">
         <v>13</v>
       </c>
-      <c r="F25" s="13">
+      <c r="F25" s="8">
         <v>6</v>
       </c>
-      <c r="G25" s="13"/>
-      <c r="H25" s="2">
+      <c r="G25" s="8"/>
+      <c r="H25" s="8">
         <v>6</v>
       </c>
-      <c r="I25" s="22"/>
-      <c r="J25" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K25" s="4">
+      <c r="I25" s="8">
+        <v>6</v>
+      </c>
+      <c r="J25" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="K25" s="10">
         <v>46015</v>
       </c>
-      <c r="L25" s="23"/>
-      <c r="M25" s="23"/>
-      <c r="N25" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="O25" s="7"/>
-      <c r="P25" s="23"/>
-      <c r="Q25" s="6" t="str">
+      <c r="L25" s="10">
+        <v>46090</v>
+      </c>
+      <c r="M25" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N25" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="O25" s="26"/>
+      <c r="P25" s="21"/>
+      <c r="Q25" s="12" t="str">
         <f>HYPERLINK("#'Vessel'!A1","Vessel")</f>
         <v>Vessel</v>
       </c>
-      <c r="R25" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="S25" s="23"/>
-      <c r="T25" s="23"/>
+      <c r="R25" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="S25" s="21"/>
+      <c r="T25" s="25" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="26" spans="1:20" ht="31.5">
       <c r="A26" s="22">
@@ -2245,7 +2294,7 @@
         <v>19</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D26" s="13">
         <v>76</v>
@@ -2457,7 +2506,9 @@
       </c>
       <c r="L30" s="23"/>
       <c r="M30" s="23"/>
-      <c r="N30" s="23"/>
+      <c r="N30" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="O30" s="25"/>
       <c r="P30" s="23"/>
       <c r="Q30" s="6" t="str">
@@ -2505,13 +2556,11 @@
       <c r="L31" s="10">
         <v>46063</v>
       </c>
-      <c r="M31" s="10" t="s">
-        <v>24</v>
-      </c>
+      <c r="M31" s="21"/>
       <c r="N31" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="O31" s="43"/>
+      <c r="O31" s="38"/>
       <c r="P31" s="21"/>
       <c r="Q31" s="12" t="str">
         <f>HYPERLINK("#'Stuffing Master'!A1","Stuffing Master")</f>
@@ -2522,7 +2571,7 @@
       </c>
       <c r="S31" s="21"/>
       <c r="T31" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:20" ht="31.5">
@@ -2676,7 +2725,7 @@
         <v>19</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D35" s="13">
         <v>14</v>
@@ -2716,44 +2765,44 @@
       <c r="T35" s="23"/>
     </row>
     <row r="36" spans="1:20" ht="31.5">
-      <c r="A36" s="40">
+      <c r="A36" s="22">
         <v>35</v>
       </c>
-      <c r="B36" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" s="30">
-        <v>115</v>
-      </c>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="31"/>
-      <c r="J36" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="K36" s="32">
-        <v>46041</v>
-      </c>
-      <c r="L36" s="31"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="O36" s="33"/>
-      <c r="P36" s="31"/>
-      <c r="Q36" s="50" t="str">
-        <f>HYPERLINK("#'Shipment Reg-Shipment'!A1","Shipment Reg-Shipment")</f>
-        <v>Shipment Reg-Shipment</v>
-      </c>
-      <c r="R36" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="S36" s="31"/>
+      <c r="B36" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D36" s="13">
+        <v>15</v>
+      </c>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
+      <c r="I36" s="13"/>
+      <c r="J36" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K36" s="14">
+        <v>46052</v>
+      </c>
+      <c r="L36" s="27"/>
+      <c r="M36" s="27"/>
+      <c r="N36" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O36" s="28"/>
+      <c r="P36" s="36"/>
+      <c r="Q36" s="29" t="str">
+        <f>HYPERLINK("#'CHA Port Master'!A1","CHA Port Master")</f>
+        <v>CHA Port Master</v>
+      </c>
+      <c r="R36" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="S36" s="23"/>
       <c r="T36" s="23"/>
     </row>
     <row r="37" spans="1:20" ht="31.5">
@@ -2764,7 +2813,7 @@
         <v>19</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D37" s="13">
         <v>15</v>
@@ -2778,7 +2827,7 @@
         <v>20</v>
       </c>
       <c r="K37" s="14">
-        <v>46052</v>
+        <v>46053</v>
       </c>
       <c r="L37" s="27"/>
       <c r="M37" s="27"/>
@@ -2786,10 +2835,10 @@
         <v>22</v>
       </c>
       <c r="O37" s="28"/>
-      <c r="P37" s="41"/>
+      <c r="P37" s="36"/>
       <c r="Q37" s="29" t="str">
-        <f>HYPERLINK("#'CHA Port Master'!A1","CHA Port Master")</f>
-        <v>CHA Port Master</v>
+        <f>HYPERLINK("#'Transporter Master'!A1","Transporter Master")</f>
+        <v>Transporter Master</v>
       </c>
       <c r="R37" s="14" t="s">
         <v>23</v>
@@ -2805,10 +2854,10 @@
         <v>19</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D38" s="13">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E38" s="13"/>
       <c r="F38" s="13"/>
@@ -2819,7 +2868,7 @@
         <v>20</v>
       </c>
       <c r="K38" s="14">
-        <v>46053</v>
+        <v>46055</v>
       </c>
       <c r="L38" s="27"/>
       <c r="M38" s="27"/>
@@ -2827,10 +2876,10 @@
         <v>22</v>
       </c>
       <c r="O38" s="28"/>
-      <c r="P38" s="41"/>
+      <c r="P38" s="36"/>
       <c r="Q38" s="29" t="str">
-        <f>HYPERLINK("#'Transporter Master'!A1","Transporter Master")</f>
-        <v>Transporter Master</v>
+        <f>HYPERLINK("#'Drawback Schedule'!A1","Drawback Schedule")</f>
+        <v>Drawback Schedule</v>
       </c>
       <c r="R38" s="14" t="s">
         <v>23</v>
@@ -2846,10 +2895,10 @@
         <v>19</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D39" s="13">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
@@ -2860,7 +2909,7 @@
         <v>20</v>
       </c>
       <c r="K39" s="14">
-        <v>46055</v>
+        <v>46057</v>
       </c>
       <c r="L39" s="27"/>
       <c r="M39" s="27"/>
@@ -2868,10 +2917,10 @@
         <v>22</v>
       </c>
       <c r="O39" s="28"/>
-      <c r="P39" s="41"/>
+      <c r="P39" s="36"/>
       <c r="Q39" s="29" t="str">
-        <f>HYPERLINK("#'Drawback Schedule'!A1","Drawback Schedule")</f>
-        <v>Drawback Schedule</v>
+        <f>HYPERLINK("#'EDI-Country'!A1","EDI-Country")</f>
+        <v>EDI-Country</v>
       </c>
       <c r="R39" s="14" t="s">
         <v>23</v>
@@ -2887,10 +2936,10 @@
         <v>19</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D40" s="13">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E40" s="13"/>
       <c r="F40" s="13"/>
@@ -2909,10 +2958,10 @@
         <v>22</v>
       </c>
       <c r="O40" s="28"/>
-      <c r="P40" s="41"/>
+      <c r="P40" s="36"/>
       <c r="Q40" s="29" t="str">
-        <f>HYPERLINK("#'EDI-Country'!A1","EDI-Country")</f>
-        <v>EDI-Country</v>
+        <f>HYPERLINK("#'Licence Master New'!A1","Licence Master New")</f>
+        <v>Licence Master New</v>
       </c>
       <c r="R40" s="14" t="s">
         <v>23</v>
@@ -2928,10 +2977,10 @@
         <v>19</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D41" s="13">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="E41" s="13"/>
       <c r="F41" s="13"/>
@@ -2942,7 +2991,7 @@
         <v>20</v>
       </c>
       <c r="K41" s="14">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="L41" s="27"/>
       <c r="M41" s="27"/>
@@ -2950,10 +2999,10 @@
         <v>22</v>
       </c>
       <c r="O41" s="28"/>
-      <c r="P41" s="41"/>
+      <c r="P41" s="36"/>
       <c r="Q41" s="29" t="str">
-        <f>HYPERLINK("#'Licence Master New'!A1","Licence Master New")</f>
-        <v>Licence Master New</v>
+        <f>HYPERLINK("#'eSanchit Code'!A1","eSanchit Code")</f>
+        <v>eSanchit Code</v>
       </c>
       <c r="R41" s="14" t="s">
         <v>23</v>
@@ -2969,10 +3018,10 @@
         <v>19</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D42" s="13">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E42" s="13"/>
       <c r="F42" s="13"/>
@@ -2983,7 +3032,7 @@
         <v>20</v>
       </c>
       <c r="K42" s="14">
-        <v>46058</v>
+        <v>46059</v>
       </c>
       <c r="L42" s="27"/>
       <c r="M42" s="27"/>
@@ -2991,10 +3040,10 @@
         <v>22</v>
       </c>
       <c r="O42" s="28"/>
-      <c r="P42" s="41"/>
+      <c r="P42" s="36"/>
       <c r="Q42" s="29" t="str">
-        <f>HYPERLINK("#'eSanchit Code'!A1","eSanchit Code")</f>
-        <v>eSanchit Code</v>
+        <f>HYPERLINK("#'CESS Schedule Master'!A1","CESS Schedule Master")</f>
+        <v>CESS Schedule Master</v>
       </c>
       <c r="R42" s="14" t="s">
         <v>23</v>
@@ -3010,10 +3059,10 @@
         <v>19</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D43" s="13">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E43" s="13"/>
       <c r="F43" s="13"/>
@@ -3024,7 +3073,7 @@
         <v>20</v>
       </c>
       <c r="K43" s="14">
-        <v>46059</v>
+        <v>46060</v>
       </c>
       <c r="L43" s="27"/>
       <c r="M43" s="27"/>
@@ -3032,10 +3081,10 @@
         <v>22</v>
       </c>
       <c r="O43" s="28"/>
-      <c r="P43" s="41"/>
+      <c r="P43" s="36"/>
       <c r="Q43" s="29" t="str">
-        <f>HYPERLINK("#'CESS Schedule Master'!A1","CESS Schedule Master")</f>
-        <v>CESS Schedule Master</v>
+        <f>HYPERLINK("#'Rodtep Master'!A1","Rodtep Master")</f>
+        <v>Rodtep Master</v>
       </c>
       <c r="R43" s="14" t="s">
         <v>23</v>
@@ -3051,10 +3100,10 @@
         <v>19</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D44" s="13">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
@@ -3065,7 +3114,7 @@
         <v>20</v>
       </c>
       <c r="K44" s="14">
-        <v>46060</v>
+        <v>46062</v>
       </c>
       <c r="L44" s="27"/>
       <c r="M44" s="27"/>
@@ -3073,10 +3122,10 @@
         <v>22</v>
       </c>
       <c r="O44" s="28"/>
-      <c r="P44" s="41"/>
+      <c r="P44" s="36"/>
       <c r="Q44" s="29" t="str">
-        <f>HYPERLINK("#'Rodtep Master'!A1","Rodtep Master")</f>
-        <v>Rodtep Master</v>
+        <f>HYPERLINK("#'Vehicle Owner Master'!A1","Vehicle Owner Master")</f>
+        <v>Vehicle Owner Master</v>
       </c>
       <c r="R44" s="14" t="s">
         <v>23</v>
@@ -3092,32 +3141,32 @@
         <v>19</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D45" s="13">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E45" s="23"/>
       <c r="F45" s="23"/>
       <c r="G45" s="23"/>
-      <c r="H45" s="13"/>
-      <c r="I45" s="13"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
       <c r="J45" s="14" t="s">
         <v>20</v>
       </c>
       <c r="K45" s="14">
-        <v>46062</v>
-      </c>
-      <c r="L45" s="27"/>
-      <c r="M45" s="27"/>
+        <v>46063</v>
+      </c>
+      <c r="L45" s="23"/>
+      <c r="M45" s="23"/>
       <c r="N45" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="O45" s="28"/>
-      <c r="P45" s="41"/>
+      <c r="O45" s="25"/>
+      <c r="P45" s="23"/>
       <c r="Q45" s="29" t="str">
-        <f>HYPERLINK("#'Vehicle Owner Master'!A1","Vehicle Owner Master")</f>
-        <v>Vehicle Owner Master</v>
+        <f>HYPERLINK("#'Item Template Master'!A1","Item Template Master")</f>
+        <v>Item Template Master</v>
       </c>
       <c r="R45" s="14" t="s">
         <v>23</v>
@@ -3133,7 +3182,7 @@
         <v>19</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D46" s="13">
         <v>26</v>
@@ -3147,7 +3196,7 @@
         <v>20</v>
       </c>
       <c r="K46" s="14">
-        <v>46063</v>
+        <v>46064</v>
       </c>
       <c r="L46" s="23"/>
       <c r="M46" s="23"/>
@@ -3157,8 +3206,8 @@
       <c r="O46" s="25"/>
       <c r="P46" s="23"/>
       <c r="Q46" s="29" t="str">
-        <f>HYPERLINK("#'Item Template Master'!A1","Item Template Master")</f>
-        <v>Item Template Master</v>
+        <f>HYPERLINK("#'ROSL DBK'!A1","ROSL DBK")</f>
+        <v>ROSL DBK</v>
       </c>
       <c r="R46" s="14" t="s">
         <v>23</v>
@@ -3173,10 +3222,10 @@
         <v>19</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D47" s="13">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E47" s="23"/>
       <c r="F47" s="23"/>
@@ -3187,7 +3236,7 @@
         <v>20</v>
       </c>
       <c r="K47" s="14">
-        <v>46064</v>
+        <v>46066</v>
       </c>
       <c r="L47" s="23"/>
       <c r="M47" s="23"/>
@@ -3197,61 +3246,62 @@
       <c r="O47" s="25"/>
       <c r="P47" s="23"/>
       <c r="Q47" s="29" t="str">
-        <f>HYPERLINK("#'ROSL DBK'!A1","ROSL DBK")</f>
-        <v>ROSL DBK</v>
-      </c>
-      <c r="R47" s="14" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="48" spans="1:20" ht="31.5">
-      <c r="A48" s="22">
-        <v>47</v>
-      </c>
-      <c r="B48" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C48" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D48" s="13">
-        <v>29</v>
-      </c>
-      <c r="E48" s="23"/>
-      <c r="F48" s="23"/>
-      <c r="G48" s="23"/>
-      <c r="H48" s="23"/>
-      <c r="I48" s="23"/>
-      <c r="J48" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="K48" s="14">
-        <v>46066</v>
-      </c>
-      <c r="L48" s="23"/>
-      <c r="M48" s="23"/>
-      <c r="N48" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="O48" s="25"/>
-      <c r="P48" s="23"/>
-      <c r="Q48" s="29" t="str">
         <f>HYPERLINK("#'Licence Master'!A1","Licence Master")</f>
         <v>Licence Master</v>
       </c>
-      <c r="R48" s="14" t="s">
-        <v>23</v>
-      </c>
+      <c r="R47" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" ht="31.5">
+      <c r="A48" s="40">
+        <v>47</v>
+      </c>
+      <c r="B48" s="41" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="D48" s="41">
+        <v>115</v>
+      </c>
+      <c r="E48" s="42"/>
+      <c r="F48" s="42"/>
+      <c r="G48" s="42"/>
+      <c r="H48" s="42"/>
+      <c r="I48" s="42"/>
+      <c r="J48" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="K48" s="43">
+        <v>46041</v>
+      </c>
+      <c r="L48" s="42"/>
+      <c r="M48" s="42"/>
+      <c r="N48" s="43" t="s">
+        <v>22</v>
+      </c>
+      <c r="O48" s="44"/>
+      <c r="P48" s="42"/>
+      <c r="Q48" s="45" t="str">
+        <f>HYPERLINK("#'Shipment Reg-Shipment'!A1","Shipment Reg-Shipment")</f>
+        <v>Shipment Reg-Shipment</v>
+      </c>
+      <c r="R48" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="S48" s="46"/>
     </row>
     <row r="49" spans="1:18" ht="31.5">
-      <c r="A49" s="22">
+      <c r="A49" s="24">
         <v>48</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D49" s="13">
         <v>94</v>
@@ -3270,9 +3320,9 @@
       <c r="L49" s="27"/>
       <c r="M49" s="27"/>
       <c r="N49" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="O49" s="51"/>
+        <v>22</v>
+      </c>
+      <c r="O49" s="39"/>
       <c r="P49" s="27"/>
       <c r="Q49" s="6" t="str">
         <f>HYPERLINK("#'Ledger Account'!A1","Ledger Account")</f>
@@ -3287,10 +3337,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C50" s="13" t="s">
         <v>84</v>
-      </c>
-      <c r="C50" s="13" t="s">
-        <v>86</v>
       </c>
       <c r="D50" s="13">
         <v>45</v>
@@ -3311,7 +3361,7 @@
       <c r="N50" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="O50" s="51"/>
+      <c r="O50" s="39"/>
       <c r="P50" s="27"/>
       <c r="Q50" s="6" t="str">
         <f>HYPERLINK("#'GST Charges'!A1","GST Charges")</f>
@@ -3329,15 +3379,21 @@
         <v>39</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D51" s="2">
         <v>11</v>
       </c>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
+      <c r="E51" s="2">
+        <v>7</v>
+      </c>
+      <c r="F51" s="2">
+        <v>4</v>
+      </c>
       <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
+      <c r="H51" s="2">
+        <v>4</v>
+      </c>
       <c r="I51" s="2"/>
       <c r="J51" s="14" t="s">
         <v>20</v>
@@ -3365,10 +3421,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D52" s="2">
         <v>12</v>
@@ -3404,13 +3460,13 @@
         <v>52</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D53" s="2">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
@@ -3435,6 +3491,279 @@
         <v>Charge Rules</v>
       </c>
       <c r="R53" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" ht="31.5">
+      <c r="A54" s="24">
+        <v>53</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D54" s="13">
+        <v>21</v>
+      </c>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="13"/>
+      <c r="I54" s="13"/>
+      <c r="J54" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K54" s="14">
+        <v>46087</v>
+      </c>
+      <c r="L54" s="23"/>
+      <c r="M54" s="23"/>
+      <c r="N54" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O54" s="7"/>
+      <c r="P54" s="2"/>
+      <c r="Q54" s="6" t="str">
+        <f>HYPERLINK("#'Item Master'!A1","Item Master")</f>
+        <v>Item Master</v>
+      </c>
+      <c r="R54" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" ht="31.5">
+      <c r="A55" s="24">
+        <v>54</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D55" s="15">
+        <v>4</v>
+      </c>
+      <c r="E55" s="2"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="47"/>
+      <c r="J55" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K55" s="14">
+        <v>46088</v>
+      </c>
+      <c r="L55" s="23"/>
+      <c r="M55" s="23"/>
+      <c r="N55" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O55" s="7"/>
+      <c r="P55" s="48"/>
+      <c r="Q55" s="6" t="str">
+        <f>HYPERLINK("#'Division Mapping'!A1","Division Mapping")</f>
+        <v>Division Mapping</v>
+      </c>
+      <c r="R55" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" ht="31.5">
+      <c r="A56" s="22">
+        <v>55</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D56" s="15">
+        <v>29</v>
+      </c>
+      <c r="E56" s="2"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
+      <c r="I56" s="22"/>
+      <c r="J56" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K56" s="14">
+        <v>46088</v>
+      </c>
+      <c r="L56" s="23"/>
+      <c r="M56" s="23"/>
+      <c r="N56" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O56" s="7"/>
+      <c r="P56" s="23"/>
+      <c r="Q56" s="6" t="str">
+        <f>HYPERLINK("#'TDS Party'!A1","TDS Party")</f>
+        <v>TDS Party</v>
+      </c>
+      <c r="R56" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" ht="31.5">
+      <c r="A57" s="22">
+        <v>56</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D57" s="13">
+        <v>18</v>
+      </c>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="24"/>
+      <c r="J57" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K57" s="14">
+        <v>46091</v>
+      </c>
+      <c r="L57" s="23"/>
+      <c r="M57" s="23"/>
+      <c r="N57" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O57" s="7"/>
+      <c r="P57" s="23"/>
+      <c r="Q57" s="6" t="str">
+        <f>HYPERLINK("#'SAC Master'!A1","SAC Master")</f>
+        <v>SAC Master</v>
+      </c>
+      <c r="R57" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" ht="31.5">
+      <c r="A58" s="22">
+        <v>57</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D58" s="13">
+        <v>13</v>
+      </c>
+      <c r="E58" s="13"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="13"/>
+      <c r="I58" s="24"/>
+      <c r="J58" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K58" s="14">
+        <v>46092</v>
+      </c>
+      <c r="L58" s="23"/>
+      <c r="M58" s="23"/>
+      <c r="N58" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O58" s="7"/>
+      <c r="P58" s="23"/>
+      <c r="Q58" s="6" t="str">
+        <f>HYPERLINK("#'Depreciation Rates Master'!A1","Depreciation Rates Master")</f>
+        <v>Depreciation Rates Master</v>
+      </c>
+      <c r="R58" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" ht="31.5">
+      <c r="A59" s="22">
+        <v>58</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="D59" s="13">
+        <v>9</v>
+      </c>
+      <c r="E59" s="13"/>
+      <c r="F59" s="13"/>
+      <c r="G59" s="13"/>
+      <c r="H59" s="13"/>
+      <c r="I59" s="24"/>
+      <c r="J59" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K59" s="14">
+        <v>46093</v>
+      </c>
+      <c r="L59" s="23"/>
+      <c r="M59" s="23"/>
+      <c r="N59" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O59" s="7"/>
+      <c r="P59" s="23"/>
+      <c r="Q59" s="6" t="str">
+        <f>HYPERLINK("#'Merge Accounts'!A1","Merge Accounts")</f>
+        <v>Merge Accounts</v>
+      </c>
+      <c r="R59" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" ht="31.5">
+      <c r="A60" s="22">
+        <v>59</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C60" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D60" s="13">
+        <v>18</v>
+      </c>
+      <c r="E60" s="13"/>
+      <c r="F60" s="13"/>
+      <c r="G60" s="13"/>
+      <c r="H60" s="13"/>
+      <c r="I60" s="24"/>
+      <c r="J60" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="K60" s="14">
+        <v>46093</v>
+      </c>
+      <c r="L60" s="23"/>
+      <c r="M60" s="23"/>
+      <c r="N60" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O60" s="7"/>
+      <c r="P60" s="23"/>
+      <c r="Q60" s="6" t="str">
+        <f>HYPERLINK("#'Receipt Voucher'!A1","Receipt Voucher")</f>
+        <v>Receipt Voucher</v>
+      </c>
+      <c r="R60" s="14" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>